<commit_message>
Add return Uber, Charge Source column, and receipt packet for Westin La Paloma ER
- Archive the missing return Uber receipt (Westin La Paloma -> TUS Airport,
  8/21, $60.24) found via a second Inbox Receipts pass; drop a duplicate of
  the already-archived outbound Uber receipt
- Add the Charge Source column to the ER build script (previously only on
  Mohonk's), rebuild the xlsx with the new Uber line - total now $1,156.88
- Build the receipt packet PDF (14 pages, chronological, letterhead-mounted
  physical receipts) via a new Python/pypdf pipeline mirroring the Mohonk
  build; install Python 3.12 + pypdf/pillow/pymupdf to support it
- Update the trip receipt log and todo.md to reflect both changes

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/travel/trips/2026-08-16_2026-08-21_westin-la-paloma-expense-report.xlsx
+++ b/travel/trips/2026-08-16_2026-08-21_westin-la-paloma-expense-report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Documents\Group-2\travel\trips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{90A134E9-B2B0-4C20-892A-04419D1EDCDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5CDED743-CB9F-4F3F-B312-C98B53FA2E9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1480" yWindow="1480" windowWidth="14400" windowHeight="8170" xr2:uid="{AB226A7D-3AA8-4D08-956B-C38E270B2EAC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{70C05564-C6FE-4CA7-9D27-E23745724B8E}"/>
   </bookViews>
   <sheets>
     <sheet name="ER Detail" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="46">
   <si>
     <t>UNIFOCUS EXPENSE REPORT  |  Westin La Paloma - HMAlpha Onsite Training</t>
   </si>
@@ -87,6 +87,9 @@
     <t>Charge Code</t>
   </si>
   <si>
+    <t>Charge Source</t>
+  </si>
+  <si>
     <t>PERSONAL</t>
   </si>
   <si>
@@ -102,6 +105,9 @@
     <t/>
   </si>
   <si>
+    <t>Visa -2674</t>
+  </si>
+  <si>
     <t>Marczyk's Fine Foods, Denver Airport (DEN layover, outbound) - lunch; Visa -2674</t>
   </si>
   <si>
@@ -112,6 +118,9 @@
   </si>
   <si>
     <t>Taxi/Train/Bus</t>
+  </si>
+  <si>
+    <t>Uber (driver Scott), Westin La Paloma -&gt; TUS Airport, 16.08 mi/40 min - UberX .15 + Airport Surcharge .00 + Booking Fee .79 + Wait Time .30 + tip .00; Visa -2674</t>
   </si>
   <si>
     <t>Marczyk's Fine Foods, Denver Airport (DEN layover, return) - lunch: Mediterranean Chicken Wrap, Genoa/Prosciutto Snack Pack, Marion Milk Choco Sea Salt, Essentia Water; Visa -2674</t>
@@ -276,7 +285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -288,6 +297,9 @@
     <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -318,10 +330,10 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -660,11 +672,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37396A75-CF43-49DE-BCC7-17E14D83C656}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1889B323-3700-46ED-B45B-176116843F7B}">
   <sheetPr>
     <tabColor rgb="FFB6752E"/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6328125" customWidth="1"/>
@@ -677,9 +689,11 @@
     <col min="8" max="8" width="12.6328125" customWidth="1"/>
     <col min="9" max="9" width="30.6328125" customWidth="1"/>
     <col min="10" max="10" width="10.6328125" customWidth="1"/>
+    <col min="11" max="11" width="3.6328125" customWidth="1"/>
+    <col min="12" max="12" width="20.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -692,8 +706,10 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -713,7 +729,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
@@ -744,403 +760,487 @@
       <c r="J4" s="6" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="7">
+      <c r="K4" s="7"/>
+      <c r="L4" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5" s="8">
         <v>46250</v>
       </c>
-      <c r="B5" s="8" t="str">
+      <c r="B5" s="9" t="str">
         <f>TEXT(A5,"ddd")</f>
         <v>Sun</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="10">
         <v>528.20000000000005</v>
       </c>
-      <c r="D5" s="10">
-        <v>1</v>
-      </c>
-      <c r="E5" s="9">
+      <c r="D5" s="11">
+        <v>1</v>
+      </c>
+      <c r="E5" s="10">
         <f>C5*D5</f>
         <v>528.20000000000005</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="11" t="s">
+      <c r="F5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="G5" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="H5" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="12" t="s">
+      <c r="I5" s="12" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="13">
+      <c r="J5" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A6" s="14">
         <v>46250</v>
       </c>
-      <c r="B6" s="14" t="str">
+      <c r="B6" s="15" t="str">
         <f>TEXT(A6,"ddd")</f>
         <v>Sun</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="16">
         <v>31.02</v>
       </c>
-      <c r="D6" s="16">
-        <v>1</v>
-      </c>
-      <c r="E6" s="15">
+      <c r="D6" s="17">
+        <v>1</v>
+      </c>
+      <c r="E6" s="16">
         <f>C6*D6</f>
         <v>31.02</v>
       </c>
-      <c r="F6" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="17" t="s">
+      <c r="F6" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="K6" s="12"/>
+      <c r="L6" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="J6" s="18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="7">
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7" s="8">
         <v>46250</v>
       </c>
-      <c r="B7" s="8" t="str">
+      <c r="B7" s="9" t="str">
         <f>TEXT(A7,"ddd")</f>
         <v>Sun</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>46.73</v>
       </c>
-      <c r="D7" s="10">
-        <v>1</v>
-      </c>
-      <c r="E7" s="9">
+      <c r="D7" s="11">
+        <v>1</v>
+      </c>
+      <c r="E7" s="10">
         <f>C7*D7</f>
         <v>46.73</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J7" s="12" t="s">
+      <c r="F7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="12" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="13">
+      <c r="J7" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A8" s="14">
         <v>46255</v>
       </c>
-      <c r="B8" s="14" t="str">
+      <c r="B8" s="15" t="str">
         <f>TEXT(A8,"ddd")</f>
         <v>Fri</v>
       </c>
-      <c r="C8" s="15">
-        <v>37.49</v>
-      </c>
-      <c r="D8" s="16">
-        <v>1</v>
-      </c>
-      <c r="E8" s="15">
+      <c r="C8" s="16">
+        <v>60.24</v>
+      </c>
+      <c r="D8" s="17">
+        <v>1</v>
+      </c>
+      <c r="E8" s="16">
         <f>C8*D8</f>
-        <v>37.49</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="14" t="s">
+        <v>60.24</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="K8" s="12"/>
+      <c r="L8" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="J8" s="18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="7">
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9" s="8">
         <v>46255</v>
       </c>
-      <c r="B9" s="8" t="str">
+      <c r="B9" s="9" t="str">
         <f>TEXT(A9,"ddd")</f>
         <v>Fri</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="10">
+        <v>37.49</v>
+      </c>
+      <c r="D9" s="11">
+        <v>1</v>
+      </c>
+      <c r="E9" s="10">
+        <f>C9*D9</f>
+        <v>37.49</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A10" s="14">
+        <v>46255</v>
+      </c>
+      <c r="B10" s="15" t="str">
+        <f>TEXT(A10,"ddd")</f>
+        <v>Fri</v>
+      </c>
+      <c r="C10" s="16">
         <v>453.2</v>
       </c>
-      <c r="D9" s="10">
-        <v>1</v>
-      </c>
-      <c r="E9" s="9">
-        <f>C9*D9</f>
+      <c r="D10" s="17">
+        <v>1</v>
+      </c>
+      <c r="E10" s="16">
+        <f>C10*D10</f>
         <v>453.2</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="I9" s="11" t="s">
+      <c r="F10" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="12" t="s">
+      <c r="I10" s="18" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14" t="str">
-        <f>IF(A10="","",TEXT(A10,"ddd"))</f>
-        <v/>
-      </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="16">
-        <v>1</v>
-      </c>
-      <c r="E10" s="15">
-        <f>C10*D10</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="20"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="7"/>
-      <c r="B11" s="8" t="str">
+      <c r="J10" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="K10" s="12"/>
+      <c r="L10" s="18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11" s="8"/>
+      <c r="B11" s="9" t="str">
         <f>IF(A11="","",TEXT(A11,"ddd"))</f>
         <v/>
       </c>
-      <c r="C11" s="21"/>
-      <c r="D11" s="10">
-        <v>1</v>
-      </c>
-      <c r="E11" s="9">
+      <c r="C11" s="20"/>
+      <c r="D11" s="11">
+        <v>1</v>
+      </c>
+      <c r="E11" s="10">
         <f>C11*D11</f>
         <v>0</v>
       </c>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="22"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14" t="str">
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="21"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" s="14"/>
+      <c r="B12" s="15" t="str">
         <f>IF(A12="","",TEXT(A12,"ddd"))</f>
         <v/>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="16">
-        <v>1</v>
-      </c>
-      <c r="E12" s="15">
+      <c r="C12" s="22"/>
+      <c r="D12" s="17">
+        <v>1</v>
+      </c>
+      <c r="E12" s="16">
         <f>C12*D12</f>
         <v>0</v>
       </c>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="20"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="7"/>
-      <c r="B13" s="8" t="str">
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="18"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13" s="8"/>
+      <c r="B13" s="9" t="str">
         <f>IF(A13="","",TEXT(A13,"ddd"))</f>
         <v/>
       </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="10">
-        <v>1</v>
-      </c>
-      <c r="E13" s="9">
+      <c r="C13" s="20"/>
+      <c r="D13" s="11">
+        <v>1</v>
+      </c>
+      <c r="E13" s="10">
         <f>C13*D13</f>
         <v>0</v>
       </c>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="22"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14" t="str">
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="21"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A14" s="14"/>
+      <c r="B14" s="15" t="str">
         <f>IF(A14="","",TEXT(A14,"ddd"))</f>
         <v/>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="16">
-        <v>1</v>
-      </c>
-      <c r="E14" s="15">
+      <c r="C14" s="22"/>
+      <c r="D14" s="17">
+        <v>1</v>
+      </c>
+      <c r="E14" s="16">
         <f>C14*D14</f>
         <v>0</v>
       </c>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="20"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8" t="str">
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="18"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A15" s="8"/>
+      <c r="B15" s="9" t="str">
         <f>IF(A15="","",TEXT(A15,"ddd"))</f>
         <v/>
       </c>
-      <c r="C15" s="21"/>
-      <c r="D15" s="10">
-        <v>1</v>
-      </c>
-      <c r="E15" s="9">
+      <c r="C15" s="20"/>
+      <c r="D15" s="11">
+        <v>1</v>
+      </c>
+      <c r="E15" s="10">
         <f>C15*D15</f>
         <v>0</v>
       </c>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="22"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14" t="str">
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="21"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A16" s="14"/>
+      <c r="B16" s="15" t="str">
         <f>IF(A16="","",TEXT(A16,"ddd"))</f>
         <v/>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="16">
-        <v>1</v>
-      </c>
-      <c r="E16" s="15">
+      <c r="C16" s="22"/>
+      <c r="D16" s="17">
+        <v>1</v>
+      </c>
+      <c r="E16" s="16">
         <f>C16*D16</f>
         <v>0</v>
       </c>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="20"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="7"/>
-      <c r="B17" s="8" t="str">
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="18"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A17" s="8"/>
+      <c r="B17" s="9" t="str">
         <f>IF(A17="","",TEXT(A17,"ddd"))</f>
         <v/>
       </c>
-      <c r="C17" s="21"/>
-      <c r="D17" s="10">
-        <v>1</v>
-      </c>
-      <c r="E17" s="9">
+      <c r="C17" s="20"/>
+      <c r="D17" s="11">
+        <v>1</v>
+      </c>
+      <c r="E17" s="10">
         <f>C17*D17</f>
         <v>0</v>
       </c>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="22"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14" t="str">
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="21"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A18" s="14"/>
+      <c r="B18" s="15" t="str">
         <f>IF(A18="","",TEXT(A18,"ddd"))</f>
         <v/>
       </c>
-      <c r="C18" s="19"/>
-      <c r="D18" s="16">
-        <v>1</v>
-      </c>
-      <c r="E18" s="15">
+      <c r="C18" s="22"/>
+      <c r="D18" s="17">
+        <v>1</v>
+      </c>
+      <c r="E18" s="16">
         <f>C18*D18</f>
         <v>0</v>
       </c>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="20"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="7"/>
-      <c r="B19" s="8" t="str">
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="18"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A19" s="8"/>
+      <c r="B19" s="9" t="str">
         <f>IF(A19="","",TEXT(A19,"ddd"))</f>
         <v/>
       </c>
-      <c r="C19" s="21"/>
-      <c r="D19" s="10">
-        <v>1</v>
-      </c>
-      <c r="E19" s="9">
+      <c r="C19" s="20"/>
+      <c r="D19" s="11">
+        <v>1</v>
+      </c>
+      <c r="E19" s="10">
         <f>C19*D19</f>
         <v>0</v>
       </c>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="22"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="23"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="E20" s="25">
-        <f>SUM(E5:E19)</f>
-        <v>1096.6400000000001</v>
-      </c>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="21"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A20" s="14"/>
+      <c r="B20" s="15" t="str">
+        <f>IF(A20="","",TEXT(A20,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="C20" s="22"/>
+      <c r="D20" s="17">
+        <v>1</v>
+      </c>
+      <c r="E20" s="16">
+        <f>C20*D20</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
       <c r="J20" s="23"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="18"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A21" s="24"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="E21" s="26">
+        <f>SUM(E5:E20)</f>
+        <v>1156.8800000000001</v>
+      </c>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F19" xr:uid="{B3B2890C-BC3E-4702-A1D4-31227A3AEA5A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F20" xr:uid="{44E949A7-4982-43C1-84E1-8C75B82C9FC4}">
       <formula1>"UF,PERSONAL,OTHER"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H19" xr:uid="{01019E97-1391-4393-BF14-260AA9565606}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H20" xr:uid="{8B3D9E3C-0909-4E2F-BC56-4C2AE9E00B0D}">
       <formula1>"Air Fare,Taxi/Train/Bus,Car Rental,Gas/Tolls,Parking,Hotel,Bkfst,Lunch,Dinner,Phone/Data,Computer,Other,Postage,Misc"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1149,7 +1249,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26DDC2B3-D904-4454-AD82-A97B47B8C71C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5691728E-A851-4D7C-AF9B-42CA614B1407}">
   <sheetPr>
     <tabColor rgb="FFF0E4D6"/>
   </sheetPr>
@@ -1161,82 +1261,82 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>